<commit_message>
Embed reserved Zenodo DOI in supplement; prepare upload archive
- Supplementary_Information.xlsx (Contents sheet) and supplement/README.md now cite the
  reserved archive DOI https://doi.org/10.5281/zenodo.21459720.
- .gitignore: exclude the regenerable Zenodo upload zip.
</commit_message>
<xml_diff>
--- a/docs/manuscript/supplement/Supplementary_Information.xlsx
+++ b/docs/manuscript/supplement/Supplementary_Information.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Contents" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="TableS1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="TableS2" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="TableS3" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TableS4" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="TableS5" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="TableS6" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contents" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS3" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS4" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS5" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TableS6" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -634,7 +634,7 @@
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Large derived files (harmonized reference ~12 GB, annotated query ~9 GB, trained models, background latent z_lin, per-cell scores): available in the repository / a Zenodo deposit [DOI to be added on deposit]; regenerable via the pipeline.</t>
+          <t>Large derived files (harmonized reference ~12 GB, annotated query ~9 GB, trained models, background latent z_lin, per-cell scores): available in the repository / a Zenodo deposit https://doi.org/10.5281/zenodo.21459720; regenerable via the pipeline.</t>
         </is>
       </c>
     </row>

</xml_diff>